<commit_message>
Make product code sequential - auto increment from max code
</commit_message>
<xml_diff>
--- a/templates/importar_productos_template.xlsx
+++ b/templates/importar_productos_template.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duqueroso/Desktop/opencode-projects/control-plus/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60346398-03B0-4140-998E-608417BAFB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F30022F-8776-0548-8A3A-69839935550E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1600" yWindow="1400" windowWidth="27640" windowHeight="16680" xr2:uid="{C1719250-87E2-DB49-8C6B-072748A47088}"/>
   </bookViews>
   <sheets>
     <sheet name="importar_productos_template" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">importar_productos_template!$A$1:$A$397</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="406">
   <si>
     <t>nombre</t>
   </si>
@@ -1232,6 +1235,12 @@
   </si>
   <si>
     <t>TABLA PERIODICA GRANDE</t>
+  </si>
+  <si>
+    <t>CUADERNO COSIDO 100-2 LINK STICKER FEMENINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CINTA SATIN DORADO  2.5CM X 45MTS </t>
   </si>
 </sst>
 </file>
@@ -1766,7 +1775,18 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -6662,7 +6682,7 @@
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>52</v>
+        <v>404</v>
       </c>
       <c r="B199" s="1">
         <v>2990</v>
@@ -10319,7 +10339,7 @@
     </row>
     <row r="358" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
-        <v>204</v>
+        <v>405</v>
       </c>
       <c r="B358" s="1">
         <v>7600</v>
@@ -11238,6 +11258,10 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A397" xr:uid="{2CC4BADA-14F4-D54D-A860-0AAF5E159701}"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>